<commit_message>
ARTSU 09/2026: antecipações REDE passam para a conta 542 (Antecipação de Vendas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuER5Qcvr6tzzoyYEHJCtB
</commit_message>
<xml_diff>
--- a/artsu/2026-09/ARTSU_202609_conferencia.xlsx
+++ b/artsu/2026-09/ARTSU_202609_conferencia.xlsx
@@ -2464,7 +2464,7 @@
         <v>34</v>
       </c>
       <c r="C90" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D90" t="n">
         <v>813.41</v>
@@ -2486,7 +2486,7 @@
         <v>34</v>
       </c>
       <c r="C91" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D91" t="n">
         <v>3036.9</v>
@@ -2508,7 +2508,7 @@
         <v>34</v>
       </c>
       <c r="C92" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D92" t="n">
         <v>1068.72</v>
@@ -3038,7 +3038,7 @@
         <v>34</v>
       </c>
       <c r="C115" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D115" t="n">
         <v>177.17</v>
@@ -3060,7 +3060,7 @@
         <v>34</v>
       </c>
       <c r="C116" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D116" t="n">
         <v>178.64</v>
@@ -3082,7 +3082,7 @@
         <v>34</v>
       </c>
       <c r="C117" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D117" t="n">
         <v>786.0700000000001</v>
@@ -3126,7 +3126,7 @@
         <v>34</v>
       </c>
       <c r="C119" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D119" t="n">
         <v>121.97</v>
@@ -3148,7 +3148,7 @@
         <v>34</v>
       </c>
       <c r="C120" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D120" t="n">
         <v>486.71</v>

</xml_diff>

<commit_message>
ARTSU 09/2026: aplica respostas da contadora (iFood 504, PJBANK 562,80 e D E L em 493)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuER5Qcvr6tzzoyYEHJCtB
</commit_message>
<xml_diff>
--- a/artsu/2026-09/ARTSU_202609_conferencia.xlsx
+++ b/artsu/2026-09/ARTSU_202609_conferencia.xlsx
@@ -570,11 +570,7 @@
           <t>PIX RECEBIDO JOAO GUSTAVO ABREU DA SILVA</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Valor acima da mensalidade habitual (3x 159,90?) - conferir</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -886,11 +882,7 @@
           <t>PIX RECEBIDO INTEGRARE RH LTDA</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Recebimento de PJ - confirmar se é mensalidade</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1056,7 +1048,7 @@
         <v>8</v>
       </c>
       <c r="C28" t="n">
-        <v>531</v>
+        <v>504</v>
       </c>
       <c r="D28" t="n">
         <v>184.03</v>
@@ -1066,11 +1058,7 @@
           <t>PIX RECEBIDO IFOOD PAGO INSTITUICAO DE PAGAMENTO</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Recebimento do iFood Pago (sem estorno no dia) - tratado como intermediador 531</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1211,7 +1199,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>357</v>
+        <v>493</v>
       </c>
       <c r="C35" t="n">
         <v>34</v>
@@ -1224,11 +1212,7 @@
           <t>PAGTO BOLETO PJBANK PAGAMENTOS</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Boleto PJBANK de valor alto p/ taxa - confirmar natureza</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1368,11 +1352,7 @@
           <t>PIX RECEBIDO ISAIAS FRANCISCO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Valor acima da mensalidade habitual - conferir</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1516,7 +1496,7 @@
         <v>8</v>
       </c>
       <c r="C48" t="n">
-        <v>531</v>
+        <v>504</v>
       </c>
       <c r="D48" t="n">
         <v>615</v>
@@ -1526,11 +1506,7 @@
           <t>PIX RECEBIDO IFOOD PAGO INSTITUICAO DE PAGAMENTO</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Recebimento do iFood Pago (sem estorno no dia) - tratado como intermediador 531</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1860,11 +1836,7 @@
           <t>PIX RECEBIDO JEFFERSON DOS SANTOS</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Valor atípico (R$ 3,00) - conferir</t>
-        </is>
-      </c>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1939,7 +1911,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>521</v>
+        <v>493</v>
       </c>
       <c r="C67" t="n">
         <v>8</v>
@@ -1952,11 +1924,7 @@
           <t>COMPRA NO DEBITO D E L DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Distribuidora - tratado como alimentação 521</t>
-        </is>
-      </c>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2022,11 +1990,7 @@
           <t>COMPRA NO DEBITO RECANTO 8</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Estabelecimento não identificado - tratado como alimentação 521</t>
-        </is>
-      </c>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2246,11 +2210,7 @@
           <t>PIX RECEBIDO ATELIE DO SORRISO ODONTOLOGIA LTDA</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Recebimento de PJ - confirmar se é mensalidade</t>
-        </is>
-      </c>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2448,11 +2408,7 @@
           <t>PREST. EMPRESTIMO FINANCIAMENTO PARC 005/006</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Duas débitos da PARC 005/006 no mesmo dia (1.381,96 + 1.975,51) - confirmar se há juros a segregar</t>
-        </is>
-      </c>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2540,11 +2496,7 @@
           <t>PREST. EMPRESTIMO FINANCIAMENTO PARC 005/006</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Duas débitos da PARC 005/006 no mesmo dia - confirmar</t>
-        </is>
-      </c>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2816,11 +2768,7 @@
           <t>PIX ENVIADO NU PAGAMENTOS SA - CARTAO</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Pix p/ Nu Pagamentos sem crédito no Nubank da Artsu - tratado como fatura de cartão 357</t>
-        </is>
-      </c>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3412,11 +3360,7 @@
           <t>PIX RECEBIDO HAMBURGUELLAS LTDA</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>Recebimento de PJ fora do padrão - confirmar natureza</t>
-        </is>
-      </c>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3592,11 +3536,7 @@
           <t>PAGTO BOLETO NU PAGAMENTOS SA - FATURA CARTAO</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>Boleto Nu Pagamentos - tratado como fatura de cartão 357</t>
-        </is>
-      </c>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3697,7 +3637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3743,33 +3683,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34</v>
+        <v>359</v>
       </c>
       <c r="C2" t="n">
-        <v>504</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>479.7</v>
+        <v>70</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO JOAO GUSTAVO ABREU DA SILVA</t>
+          <t>PIX ENVIADO MOVE ELETROMOBILIDADE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Valor acima da mensalidade habitual (3x 159,90?) - conferir</t>
+          <t>PJ nova sem classificação (eletromobilidade) - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3779,127 +3719,127 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PIX ENVIADO MOVE ELETROMOBILIDADE</t>
+          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PJ nova sem classificação (eletromobilidade) - 359 provisório</t>
+          <t>PJ nova (publicidade) - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>359</v>
       </c>
       <c r="C4" t="n">
-        <v>504</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>219.9</v>
+        <v>50</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO INTEGRARE RH LTDA</t>
+          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Recebimento de PJ - confirmar se é mensalidade</t>
+          <t>PJ nova (publicidade) - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>510</v>
       </c>
       <c r="C5" t="n">
-        <v>531</v>
+        <v>34</v>
       </c>
       <c r="D5" t="n">
-        <v>184.03</v>
+        <v>382.74</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO IFOOD PAGO INSTITUICAO DE PAGAMENTO</t>
+          <t>PAGTO BOLETO RBA CONTABILIDADE HONORARIOS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Recebimento do iFood Pago (sem estorno no dia) - tratado como intermediador 531</t>
+          <t>Boleto pago em duplicidade - estornado no mesmo dia</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C6" t="n">
         <v>34</v>
       </c>
       <c r="D6" t="n">
-        <v>562.8</v>
+        <v>35</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PAGTO BOLETO PJBANK PAGAMENTOS</t>
+          <t>PIX ENVIADO HENRIQUE TRICH (MEI 60.229.581)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Boleto PJBANK de valor alto p/ taxa - confirmar natureza</t>
+          <t>MEI novo - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>359</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>199.5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
+          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
+          <t>MEI novo - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3909,484 +3849,94 @@
         <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
+          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
+          <t>PJ nova (CT/academia) - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>359</v>
       </c>
       <c r="C9" t="n">
-        <v>504</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>489.7</v>
+        <v>465.5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO ISAIAS FRANCISCO DE OLIVEIRA JUNIOR</t>
+          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Valor acima da mensalidade habitual - conferir</t>
+          <t>MEI novo - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>359</v>
       </c>
       <c r="C10" t="n">
-        <v>531</v>
+        <v>34</v>
       </c>
       <c r="D10" t="n">
-        <v>615</v>
+        <v>6</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO IFOOD PAGO INSTITUICAO DE PAGAMENTO</t>
+          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Recebimento do iFood Pago (sem estorno no dia) - tratado como intermediador 531</t>
+          <t>PJ nova (CT/academia) - 359 provisório</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>359</v>
       </c>
       <c r="C11" t="n">
-        <v>504</v>
+        <v>34</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>237.7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PIX RECEBIDO JEFFERSON DOS SANTOS</t>
+          <t>PIX ENVIADO BODYRIT ACADEMIA E SERVICOS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Valor atípico (R$ 3,00) - conferir</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>521</v>
-      </c>
-      <c r="C12" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>COMPRA NO DEBITO D E L DISTRIBUIDORA</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Distribuidora - tratado como alimentação 521</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>521</v>
-      </c>
-      <c r="C13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" t="n">
-        <v>56.81</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>COMPRA NO DEBITO RECANTO 8</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Estabelecimento não identificado - tratado como alimentação 521</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>16/09/2026</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>8</v>
-      </c>
-      <c r="C14" t="n">
-        <v>504</v>
-      </c>
-      <c r="D14" t="n">
-        <v>190</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>PIX RECEBIDO ATELIE DO SORRISO ODONTOLOGIA LTDA</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Recebimento de PJ - confirmar se é mensalidade</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>21/09/2026</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>152</v>
-      </c>
-      <c r="C15" t="n">
-        <v>34</v>
-      </c>
-      <c r="D15" t="n">
-        <v>1381.96</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>PREST. EMPRESTIMO FINANCIAMENTO PARC 005/006</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Duas débitos da PARC 005/006 no mesmo dia (1.381,96 + 1.975,51) - confirmar se há juros a segregar</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>21/09/2026</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>152</v>
-      </c>
-      <c r="C16" t="n">
-        <v>34</v>
-      </c>
-      <c r="D16" t="n">
-        <v>1975.51</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>PREST. EMPRESTIMO FINANCIAMENTO PARC 005/006</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Duas débitos da PARC 005/006 no mesmo dia - confirmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>510</v>
-      </c>
-      <c r="C17" t="n">
-        <v>34</v>
-      </c>
-      <c r="D17" t="n">
-        <v>382.74</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>PAGTO BOLETO RBA CONTABILIDADE HONORARIOS</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Boleto pago em duplicidade - estornado no mesmo dia</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>359</v>
-      </c>
-      <c r="C18" t="n">
-        <v>34</v>
-      </c>
-      <c r="D18" t="n">
-        <v>35</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO HENRIQUE TRICH (MEI 60.229.581)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>357</v>
-      </c>
-      <c r="C19" t="n">
-        <v>34</v>
-      </c>
-      <c r="D19" t="n">
-        <v>603.96</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO NU PAGAMENTOS SA - CARTAO</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Pix p/ Nu Pagamentos sem crédito no Nubank da Artsu - tratado como fatura de cartão 357</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>359</v>
-      </c>
-      <c r="C20" t="n">
-        <v>34</v>
-      </c>
-      <c r="D20" t="n">
-        <v>199.5</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>359</v>
-      </c>
-      <c r="C21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D21" t="n">
-        <v>10</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>359</v>
-      </c>
-      <c r="C22" t="n">
-        <v>34</v>
-      </c>
-      <c r="D22" t="n">
-        <v>465.5</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>359</v>
-      </c>
-      <c r="C23" t="n">
-        <v>34</v>
-      </c>
-      <c r="D23" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>359</v>
-      </c>
-      <c r="C24" t="n">
-        <v>34</v>
-      </c>
-      <c r="D24" t="n">
-        <v>237.7</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO BODYRIT ACADEMIA E SERVICOS</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
           <t>PJ nova (academia) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>34</v>
-      </c>
-      <c r="C25" t="n">
-        <v>504</v>
-      </c>
-      <c r="D25" t="n">
-        <v>480</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>PIX RECEBIDO HAMBURGUELLAS LTDA</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Recebimento de PJ fora do padrão - confirmar natureza</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>357</v>
-      </c>
-      <c r="C26" t="n">
-        <v>34</v>
-      </c>
-      <c r="D26" t="n">
-        <v>1839.8</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>PAGTO BOLETO NU PAGAMENTOS SA - FATURA CARTAO</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Boleto Nu Pagamentos - tratado como fatura de cartão 357</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ARTSU 09/2026: recebimentos Nubank em 504, Santander em 531, antecipações em 542
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuER5Qcvr6tzzoyYEHJCtB
</commit_message>
<xml_diff>
--- a/artsu/2026-09/ARTSU_202609_conferencia.xlsx
+++ b/artsu/2026-09/ARTSU_202609_conferencia.xlsx
@@ -560,7 +560,7 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D6" t="n">
         <v>479.7</v>
@@ -784,7 +784,7 @@
         <v>34</v>
       </c>
       <c r="C16" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D16" t="n">
         <v>260</v>
@@ -850,7 +850,7 @@
         <v>34</v>
       </c>
       <c r="C19" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D19" t="n">
         <v>160</v>
@@ -872,7 +872,7 @@
         <v>34</v>
       </c>
       <c r="C20" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D20" t="n">
         <v>219.9</v>
@@ -1114,7 +1114,7 @@
         <v>34</v>
       </c>
       <c r="C31" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D31" t="n">
         <v>190</v>
@@ -1246,7 +1246,7 @@
         <v>34</v>
       </c>
       <c r="C37" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D37" t="n">
         <v>255</v>
@@ -1364,7 +1364,7 @@
         <v>8</v>
       </c>
       <c r="C42" t="n">
-        <v>531</v>
+        <v>504</v>
       </c>
       <c r="D42" t="n">
         <v>117.81</v>
@@ -1452,7 +1452,7 @@
         <v>34</v>
       </c>
       <c r="C46" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D46" t="n">
         <v>144</v>
@@ -1474,7 +1474,7 @@
         <v>34</v>
       </c>
       <c r="C47" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D47" t="n">
         <v>159.9</v>
@@ -1562,7 +1562,7 @@
         <v>34</v>
       </c>
       <c r="C51" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D51" t="n">
         <v>259.8</v>
@@ -1716,7 +1716,7 @@
         <v>34</v>
       </c>
       <c r="C58" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D58" t="n">
         <v>61.47</v>
@@ -1738,7 +1738,7 @@
         <v>34</v>
       </c>
       <c r="C59" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D59" t="n">
         <v>189.9</v>
@@ -1870,7 +1870,7 @@
         <v>34</v>
       </c>
       <c r="C65" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D65" t="n">
         <v>129</v>
@@ -2134,7 +2134,7 @@
         <v>34</v>
       </c>
       <c r="C77" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D77" t="n">
         <v>319.8</v>
@@ -2156,7 +2156,7 @@
         <v>34</v>
       </c>
       <c r="C78" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D78" t="n">
         <v>190</v>
@@ -2288,7 +2288,7 @@
         <v>34</v>
       </c>
       <c r="C84" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D84" t="n">
         <v>189.9</v>
@@ -2310,7 +2310,7 @@
         <v>34</v>
       </c>
       <c r="C85" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D85" t="n">
         <v>189.9</v>
@@ -2376,7 +2376,7 @@
         <v>34</v>
       </c>
       <c r="C88" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D88" t="n">
         <v>220</v>
@@ -2600,7 +2600,7 @@
         <v>34</v>
       </c>
       <c r="C98" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D98" t="n">
         <v>320</v>
@@ -2670,7 +2670,7 @@
         <v>34</v>
       </c>
       <c r="C101" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D101" t="n">
         <v>220</v>
@@ -3236,7 +3236,7 @@
         <v>34</v>
       </c>
       <c r="C126" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D126" t="n">
         <v>100</v>
@@ -3302,7 +3302,7 @@
         <v>34</v>
       </c>
       <c r="C129" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D129" t="n">
         <v>50</v>
@@ -3350,7 +3350,7 @@
         <v>34</v>
       </c>
       <c r="C131" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D131" t="n">
         <v>480</v>
@@ -3394,7 +3394,7 @@
         <v>34</v>
       </c>
       <c r="C133" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D133" t="n">
         <v>80</v>
@@ -3504,7 +3504,7 @@
         <v>34</v>
       </c>
       <c r="C138" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D138" t="n">
         <v>180</v>
@@ -3592,7 +3592,7 @@
         <v>34</v>
       </c>
       <c r="C142" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D142" t="n">
         <v>240</v>
@@ -3614,7 +3614,7 @@
         <v>34</v>
       </c>
       <c r="C143" t="n">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="D143" t="n">
         <v>113.94</v>

</xml_diff>

<commit_message>
ARTSU 09/2026: classifica fornecedores novos (359, 467, 493) - versão final
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuER5Qcvr6tzzoyYEHJCtB
</commit_message>
<xml_diff>
--- a/artsu/2026-09/ARTSU_202609_conferencia.xlsx
+++ b/artsu/2026-09/ARTSU_202609_conferencia.xlsx
@@ -680,11 +680,7 @@
           <t>PIX ENVIADO MOVE ELETROMOBILIDADE</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PJ nova sem classificação (eletromobilidade) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1278,11 +1274,7 @@
           <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1304,11 +1296,7 @@
           <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2619,7 +2607,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>359</v>
+        <v>493</v>
       </c>
       <c r="C99" t="n">
         <v>34</v>
@@ -2629,14 +2617,10 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>PIX ENVIADO HENRIQUE TRICH (MEI 60.229.581)</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
+          <t>PIX ENVIADO HENRIQUE TRICH CABELEIREIRO</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2777,7 +2761,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>359</v>
+        <v>493</v>
       </c>
       <c r="C106" t="n">
         <v>34</v>
@@ -2787,14 +2771,10 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
+          <t>PIX ENVIADO SERGIO DA CRUZ</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2913,7 +2893,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>359</v>
+        <v>467</v>
       </c>
       <c r="C112" t="n">
         <v>8</v>
@@ -2926,11 +2906,7 @@
           <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3115,7 +3091,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>359</v>
+        <v>493</v>
       </c>
       <c r="C121" t="n">
         <v>34</v>
@@ -3125,14 +3101,10 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
+          <t>PIX ENVIADO SERGIO DA CRUZ</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3141,7 +3113,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>359</v>
+        <v>467</v>
       </c>
       <c r="C122" t="n">
         <v>34</v>
@@ -3154,11 +3126,7 @@
           <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3321,7 +3289,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>359</v>
+        <v>467</v>
       </c>
       <c r="C130" t="n">
         <v>34</v>
@@ -3334,11 +3302,7 @@
           <t>PIX ENVIADO BODYRIT ACADEMIA E SERVICOS</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>PJ nova (academia) - 359 provisório</t>
-        </is>
-      </c>
+      <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3637,7 +3601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3683,260 +3647,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>359</v>
+        <v>510</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="D2" t="n">
-        <v>70</v>
+        <v>382.74</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PIX ENVIADO MOVE ELETROMOBILIDADE</t>
+          <t>PAGTO BOLETO RBA CONTABILIDADE HONORARIOS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PJ nova sem classificação (eletromobilidade) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>359</v>
-      </c>
-      <c r="C3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D3" t="n">
-        <v>100</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>359</v>
-      </c>
-      <c r="C4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO TUPINAMBA PUBLICIDADES</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PJ nova (publicidade) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>510</v>
-      </c>
-      <c r="C5" t="n">
-        <v>34</v>
-      </c>
-      <c r="D5" t="n">
-        <v>382.74</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PAGTO BOLETO RBA CONTABILIDADE HONORARIOS</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
           <t>Boleto pago em duplicidade - estornado no mesmo dia</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>359</v>
-      </c>
-      <c r="C6" t="n">
-        <v>34</v>
-      </c>
-      <c r="D6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO HENRIQUE TRICH (MEI 60.229.581)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>359</v>
-      </c>
-      <c r="C7" t="n">
-        <v>34</v>
-      </c>
-      <c r="D7" t="n">
-        <v>199.5</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>359</v>
-      </c>
-      <c r="C8" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>359</v>
-      </c>
-      <c r="C9" t="n">
-        <v>34</v>
-      </c>
-      <c r="D9" t="n">
-        <v>465.5</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO SERGIO DA CRUZ (MEI 53.274.851)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>MEI novo - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>359</v>
-      </c>
-      <c r="C10" t="n">
-        <v>34</v>
-      </c>
-      <c r="D10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO CT ELITE PERFORMANCE LTDA</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PJ nova (CT/academia) - 359 provisório</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>359</v>
-      </c>
-      <c r="C11" t="n">
-        <v>34</v>
-      </c>
-      <c r="D11" t="n">
-        <v>237.7</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>PIX ENVIADO BODYRIT ACADEMIA E SERVICOS</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PJ nova (academia) - 359 provisório</t>
         </is>
       </c>
     </row>

</xml_diff>